<commit_message>
Update template for Jira and Confluence URL support
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kborow437@emea.comcast.com/projects/timeline/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kborow437@emea.comcast.com/projects/chronos-cli/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14EF7CD8-1092-6E49-915C-13242E7DBA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B662BC0-4B4A-5043-B5CD-27DC8BF1EDA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680" xr2:uid="{14B44724-6ACE-2D4F-8A7C-B447217C9BD8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>Task</t>
   </si>
@@ -141,6 +141,24 @@
   </si>
   <si>
     <t>Task9</t>
+  </si>
+  <si>
+    <t>Jira Link</t>
+  </si>
+  <si>
+    <t>Confluence Link</t>
+  </si>
+  <si>
+    <t>https://confluence-wiki.com</t>
+  </si>
+  <si>
+    <t>https://jira-link2.com</t>
+  </si>
+  <si>
+    <t>https://jira-link1.com</t>
+  </si>
+  <si>
+    <t>https://confluence-wiki2.com</t>
   </si>
 </sst>
 </file>
@@ -518,16 +536,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2E9CB6-0594-D24D-A8AA-5EAD24ACFE98}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -540,8 +560,14 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -554,8 +580,11 @@
       <c r="D2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -568,8 +597,11 @@
       <c r="D3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -583,7 +615,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -597,7 +629,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -611,7 +643,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -625,7 +657,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -638,8 +670,14 @@
       <c r="D8" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -653,7 +691,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>33</v>
       </c>

</xml_diff>

<commit_message>
Added new feature to link tasks. So on highlighting, all connected tasks will highlight together
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kborow437@emea.comcast.com/projects/chronos-cli/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanand806@cable.comcast.com/work/personalProjects/chronos-cli/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B662BC0-4B4A-5043-B5CD-27DC8BF1EDA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB09D5A0-3A5F-0D4D-917B-5DA05FB996D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680" xr2:uid="{14B44724-6ACE-2D4F-8A7C-B447217C9BD8}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{14B44724-6ACE-2D4F-8A7C-B447217C9BD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
   <si>
     <t>Task</t>
   </si>
@@ -159,6 +159,18 @@
   </si>
   <si>
     <t>https://confluence-wiki2.com</t>
+  </si>
+  <si>
+    <t>Connections</t>
+  </si>
+  <si>
+    <t>RandomLink1</t>
+  </si>
+  <si>
+    <t>RandomLink2</t>
+  </si>
+  <si>
+    <t>RandomLink1;RandomLink2</t>
   </si>
 </sst>
 </file>
@@ -536,18 +548,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2E9CB6-0594-D24D-A8AA-5EAD24ACFE98}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -561,13 +574,16 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" t="s">
         <v>34</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -581,10 +597,13 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -597,11 +616,14 @@
       <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="F3" t="s">
+      <c r="E3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -614,8 +636,11 @@
       <c r="D4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -629,7 +654,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -642,8 +667,11 @@
       <c r="D6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -656,8 +684,11 @@
       <c r="D7" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -670,14 +701,14 @@
       <c r="D8" t="s">
         <v>20</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>37</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -690,8 +721,11 @@
       <c r="D9" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>33</v>
       </c>

</xml_diff>

<commit_message>
Adding new columns to template
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanand806@cable.comcast.com/work/personalProjects/chronos-cli/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB09D5A0-3A5F-0D4D-917B-5DA05FB996D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3808B0F-961A-2D44-81C0-F6188EB65F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{14B44724-6ACE-2D4F-8A7C-B447217C9BD8}"/>
+    <workbookView xWindow="36000" yWindow="-26440" windowWidth="21600" windowHeight="38400" xr2:uid="{14B44724-6ACE-2D4F-8A7C-B447217C9BD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
   <si>
     <t>Task</t>
   </si>
@@ -171,6 +171,18 @@
   </si>
   <si>
     <t>RandomLink1;RandomLink2</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Lorem ipsum dolor sit amet.</t>
+  </si>
+  <si>
+    <t>Lorem ipsum dolor sit amet consectetur adipiscing elit. Consectetur adipiscing elit quisque faucibus ex sapien vitae. Ex sapien vitae pellentesque sem placerat in id. Placerat in id cursus mi pretium tellus duis. Pretium tellus duis convallis tempus leo eu aenean.</t>
+  </si>
+  <si>
+    <t>Lorem ipsum dolor sit amet consectetur adipiscing elit quisque faucibus.</t>
   </si>
 </sst>
 </file>
@@ -548,19 +560,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2E9CB6-0594-D24D-A8AA-5EAD24ACFE98}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -577,13 +589,16 @@
         <v>40</v>
       </c>
       <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
         <v>34</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -600,10 +615,13 @@
         <v>41</v>
       </c>
       <c r="F2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -619,11 +637,11 @@
       <c r="E3" t="s">
         <v>42</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -639,8 +657,11 @@
       <c r="E4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -654,7 +675,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -671,7 +692,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -688,7 +709,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -702,13 +723,16 @@
         <v>20</v>
       </c>
       <c r="F8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" t="s">
         <v>37</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -725,7 +749,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -737,6 +761,9 @@
       </c>
       <c r="D10" t="s">
         <v>24</v>
+      </c>
+      <c r="F10" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Placement column override for task positioning
- DataLoader parses optional "Placement" column ("up"/"down") and
  computes IsAbove, falling back to Type-based default when absent
- png_generator/html_generator split sections on IsAbove instead of
  hardcoding Type == "dependency"
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanand806@cable.comcast.com/work/personalProjects/chronos-cli/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3808B0F-961A-2D44-81C0-F6188EB65F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C45268B-ACAE-0C42-B089-B9CBB0D2E423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="36000" yWindow="-26440" windowWidth="21600" windowHeight="38400" xr2:uid="{14B44724-6ACE-2D4F-8A7C-B447217C9BD8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="50">
   <si>
     <t>Task</t>
   </si>
@@ -122,9 +122,6 @@
     <t>Task2</t>
   </si>
   <si>
-    <t>Task3</t>
-  </si>
-  <si>
     <t>Task4</t>
   </si>
   <si>
@@ -137,9 +134,6 @@
     <t>Task7</t>
   </si>
   <si>
-    <t>Task8</t>
-  </si>
-  <si>
     <t>Task9</t>
   </si>
   <si>
@@ -183,6 +177,18 @@
   </si>
   <si>
     <t>Lorem ipsum dolor sit amet consectetur adipiscing elit quisque faucibus.</t>
+  </si>
+  <si>
+    <t>Placement</t>
+  </si>
+  <si>
+    <t>down</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task8 </t>
+  </si>
+  <si>
+    <t>Task3 - (Forced down)</t>
   </si>
 </sst>
 </file>
@@ -560,19 +566,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2E9CB6-0594-D24D-A8AA-5EAD24ACFE98}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -586,19 +592,22 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="G1" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -611,17 +620,17 @@
       <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="s">
-        <v>41</v>
-      </c>
       <c r="F2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -634,16 +643,16 @@
       <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
-        <v>42</v>
-      </c>
-      <c r="H3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
@@ -655,15 +664,18 @@
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+      <c r="G4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
         <v>12</v>
@@ -675,9 +687,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
         <v>15</v>
@@ -688,13 +700,13 @@
       <c r="D6" t="s">
         <v>16</v>
       </c>
-      <c r="E6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
         <v>17</v>
@@ -705,13 +717,13 @@
       <c r="D7" t="s">
         <v>18</v>
       </c>
-      <c r="E7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
         <v>19</v>
@@ -722,19 +734,19 @@
       <c r="D8" t="s">
         <v>20</v>
       </c>
-      <c r="F8" t="s">
-        <v>47</v>
-      </c>
       <c r="G8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" t="s">
         <v>37</v>
       </c>
-      <c r="H8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
         <v>21</v>
@@ -746,12 +758,15 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+      <c r="F9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
@@ -762,8 +777,8 @@
       <c r="D10" t="s">
         <v>24</v>
       </c>
-      <c r="F10" t="s">
-        <v>46</v>
+      <c r="G10" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>